<commit_message>
CA et objectifs : saisie, vue Performance, légende et synthèse (admins)
- Données réservées aux admins : get_map_data ne renvoie plus les CA et
  objectifs avec le seul code d'accès (migration + test)
- Admin : section « CA et objectifs » dans le panneau d'un commercial
  (par structure et par année, taux d'atteinte en direct)
- Carte : sélecteur d'année, CA / objectif / taux dans la légende
  (commercial ou équipe d'un manager), vue « Performance » du rouge au vert
  avec classement des commerciaux
- Onglet « Synthèse » : par commercial, manager ou structure, tri, totaux,
  export Excel
- Fichier d'exemple enrichi de CA et objectifs fictifs

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exemples/exemple-import.xlsx
+++ b/exemples/exemple-import.xlsx
@@ -789,11 +789,11 @@
       <c r="R5" t="str">
         <v/>
       </c>
-      <c r="S5" t="str">
-        <v/>
-      </c>
-      <c r="T5" t="str">
-        <v/>
+      <c r="S5">
+        <v>210000</v>
+      </c>
+      <c r="T5">
+        <v>200000</v>
       </c>
       <c r="U5" t="str">
         <v/>
@@ -1003,11 +1003,11 @@
       <c r="R7" t="str">
         <v/>
       </c>
-      <c r="S7" t="str">
-        <v/>
-      </c>
-      <c r="T7" t="str">
-        <v/>
+      <c r="S7">
+        <v>95000</v>
+      </c>
+      <c r="T7">
+        <v>180000</v>
       </c>
       <c r="U7" t="str">
         <v/>
@@ -1110,11 +1110,11 @@
       <c r="R8" t="str">
         <v/>
       </c>
-      <c r="S8" t="str">
-        <v/>
-      </c>
-      <c r="T8" t="str">
-        <v/>
+      <c r="S8">
+        <v>260000</v>
+      </c>
+      <c r="T8">
+        <v>200000</v>
       </c>
       <c r="U8" t="str">
         <v/>
@@ -1217,11 +1217,11 @@
       <c r="R9" t="str">
         <v/>
       </c>
-      <c r="S9" t="str">
-        <v/>
-      </c>
-      <c r="T9" t="str">
-        <v/>
+      <c r="S9">
+        <v>60000</v>
+      </c>
+      <c r="T9">
+        <v>140000</v>
       </c>
       <c r="U9" t="str">
         <v/>
@@ -1324,11 +1324,11 @@
       <c r="R10" t="str">
         <v/>
       </c>
-      <c r="S10" t="str">
-        <v/>
-      </c>
-      <c r="T10" t="str">
-        <v/>
+      <c r="S10">
+        <v>150000</v>
+      </c>
+      <c r="T10">
+        <v>160000</v>
       </c>
       <c r="U10" t="str">
         <v/>
@@ -1651,11 +1651,11 @@
       <c r="T14" t="str">
         <v/>
       </c>
-      <c r="U14" t="str">
-        <v/>
-      </c>
-      <c r="V14" t="str">
-        <v/>
+      <c r="U14">
+        <v>70000</v>
+      </c>
+      <c r="V14">
+        <v>60000</v>
       </c>
       <c r="W14" t="str">
         <v/>
@@ -1758,11 +1758,11 @@
       <c r="T15" t="str">
         <v/>
       </c>
-      <c r="U15" t="str">
-        <v/>
-      </c>
-      <c r="V15" t="str">
-        <v/>
+      <c r="U15">
+        <v>30000</v>
+      </c>
+      <c r="V15">
+        <v>65000</v>
       </c>
       <c r="W15" t="str">
         <v/>
@@ -1865,11 +1865,11 @@
       <c r="T16" t="str">
         <v/>
       </c>
-      <c r="U16" t="str">
-        <v/>
-      </c>
-      <c r="V16" t="str">
-        <v/>
+      <c r="U16">
+        <v>55000</v>
+      </c>
+      <c r="V16">
+        <v>70000</v>
       </c>
       <c r="W16" t="str">
         <v/>
@@ -1972,11 +1972,11 @@
       <c r="T17" t="str">
         <v/>
       </c>
-      <c r="U17" t="str">
-        <v/>
-      </c>
-      <c r="V17" t="str">
-        <v/>
+      <c r="U17">
+        <v>98000</v>
+      </c>
+      <c r="V17">
+        <v>80000</v>
       </c>
       <c r="W17" t="str">
         <v/>
@@ -2299,11 +2299,11 @@
       <c r="V20" t="str">
         <v/>
       </c>
-      <c r="W20" t="str">
-        <v/>
-      </c>
-      <c r="X20" t="str">
-        <v/>
+      <c r="W20">
+        <v>45000</v>
+      </c>
+      <c r="X20">
+        <v>50000</v>
       </c>
       <c r="Y20" t="str">
         <v/>
@@ -2519,11 +2519,11 @@
       <c r="X22" t="str">
         <v/>
       </c>
-      <c r="Y22" t="str">
-        <v/>
-      </c>
-      <c r="Z22" t="str">
-        <v/>
+      <c r="Y22">
+        <v>20000</v>
+      </c>
+      <c r="Z22">
+        <v>25000</v>
       </c>
       <c r="AA22" t="str">
         <v/>

</xml_diff>